<commit_message>
Fix invisible active-tab text, use E28 for total investment, sync sheet
The active tab's text and background were both near-white, making the
selected tab unreadable; switched the text color to the dark brand
color. Initial-investment figure now reads Main!E28 (setup cost plus a
year of running-cost reserve) instead of D28 (setup cost alone), to
match the updated model. Also synced the latest Delivery.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Delivery.xlsx
+++ b/data/Delivery.xlsx
@@ -1898,7 +1898,7 @@
   <cols>
     <col min="3" max="3" width="13.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25.85546875" customWidth="1"/>
     <col min="12" max="16" width="12.7109375" customWidth="1"/>
   </cols>
@@ -2455,8 +2455,8 @@
         <v>95045.454545454544</v>
       </c>
       <c r="E28" s="10">
-        <f>D28+D31+D32</f>
-        <v>115045.45454545454</v>
+        <f>D28-SUM(L31:L37)*12</f>
+        <v>119583.33333333333</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add ROI/payback to investment card, tax column to SyTRA table
- Compute Year-1 ROI and payback period live from the workbook
  (Initial Investment vs. Year-1 annual profit) and show them next to
  the Required Initial Investment figure.
- Add a Tax Rate column to the SyTRA revenue-share table, reading the
  now-populated Main!D56 rate.
- Fix Monthly Revenue read: the user inserted a new "Number of Orders"
  row in the Main sheet, pushing Monthly Revenue from row 15 to row
  17 - the site was silently reading order counts as dollar revenue
  for the yearly table and chart. Updated the cell reference.
- Sync the latest Delivery.xlsx (new order-count row, 10% tax rate).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Delivery.xlsx
+++ b/data/Delivery.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Delivery Business\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Delivery Business\DeliveryStudy\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
   <si>
     <t>Average order value</t>
   </si>
@@ -214,16 +214,21 @@
   </si>
   <si>
     <t>SyTRA+Tax</t>
+  </si>
+  <si>
+    <t>Number of Orders</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_([$SYP]\ * #,##0_);_([$SYP]\ * \(#,##0\);_([$SYP]\ * &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="171" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -319,14 +324,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -360,9 +366,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
     <cellStyle name="Accent3" xfId="4" builtinId="37"/>
+    <cellStyle name="Comma" xfId="5" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Input" xfId="3" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -657,181 +665,181 @@
                   <c:v>5416.6666666666679</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22154.545454545463</c:v>
+                  <c:v>20109.090909090919</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>38892.424242424255</c:v>
+                  <c:v>34801.515151515167</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>55630.303030303054</c:v>
+                  <c:v>49493.939393939421</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>72368.181818181853</c:v>
+                  <c:v>64186.363636363676</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>89106.060606060651</c:v>
+                  <c:v>78878.787878787931</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>105843.93939393945</c:v>
+                  <c:v>93571.212121212186</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>122581.81818181825</c:v>
+                  <c:v>108263.63636363644</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>139319.69696969705</c:v>
+                  <c:v>122956.0606060607</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>156057.57575757583</c:v>
+                  <c:v>137648.48484848495</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>172795.45454545462</c:v>
+                  <c:v>152340.9090909092</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>102995.45454545459</c:v>
+                  <c:v>80495.454545454646</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>145242.42424242431</c:v>
+                  <c:v>121351.51515151527</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>187489.39393939404</c:v>
+                  <c:v>162207.57575757589</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>229736.36363636376</c:v>
+                  <c:v>203063.63636363653</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>271983.33333333349</c:v>
+                  <c:v>243919.69696969714</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>314230.30303030321</c:v>
+                  <c:v>284775.75757575774</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>356477.27272727294</c:v>
+                  <c:v>325631.81818181835</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>398724.24242424266</c:v>
+                  <c:v>366487.87878787896</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>440971.21212121239</c:v>
+                  <c:v>407343.93939393957</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>483218.18181818211</c:v>
+                  <c:v>448200.00000000017</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>525465.15151515184</c:v>
+                  <c:v>489056.06060606078</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>567712.12121212156</c:v>
+                  <c:v>529912.12121212145</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>402421.21212121251</c:v>
+                  <c:v>363230.30303030327</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>486824.24242424284</c:v>
+                  <c:v>450251.51515151543</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>571227.27272727317</c:v>
+                  <c:v>537272.72727272753</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>655630.30303030345</c:v>
+                  <c:v>624293.93939393968</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>740033.33333333372</c:v>
+                  <c:v>711315.15151515184</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>824436.363636364</c:v>
+                  <c:v>798336.363636364</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>908839.39393939427</c:v>
+                  <c:v>885357.57575757615</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>993242.42424242455</c:v>
+                  <c:v>972378.78787878831</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1077645.4545454548</c:v>
+                  <c:v>1059400.0000000005</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1162048.4848484851</c:v>
+                  <c:v>1146421.2121212126</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1246451.5151515154</c:v>
+                  <c:v>1233442.4242424248</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1330854.5454545456</c:v>
+                  <c:v>1320463.6363636369</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1234719.6969696973</c:v>
+                  <c:v>1226946.9696969702</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1358304.5454545459</c:v>
+                  <c:v>1362559.0909090915</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>1481889.3939393945</c:v>
+                  <c:v>1498171.2121212129</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>1605474.2424242431</c:v>
+                  <c:v>1633783.3333333342</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>1729059.0909090918</c:v>
+                  <c:v>1769395.4545454555</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>1852643.9393939404</c:v>
+                  <c:v>1905007.5757575769</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>1976228.787878789</c:v>
+                  <c:v>2040619.6969696982</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>2099813.6363636376</c:v>
+                  <c:v>2176231.8181818193</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>2223398.4848484863</c:v>
+                  <c:v>2311843.9393939404</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>2346983.3333333349</c:v>
+                  <c:v>2447456.0606060615</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>2470568.1818181835</c:v>
+                  <c:v>2583068.1818181826</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>2594153.0303030321</c:v>
+                  <c:v>2718680.3030303037</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>2529200.0000000019</c:v>
+                  <c:v>2665754.5454545463</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>2701457.5757575775</c:v>
+                  <c:v>2854048.4848484858</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>2873715.1515151532</c:v>
+                  <c:v>3042342.4242424252</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>3045972.7272727289</c:v>
+                  <c:v>3230636.3636363647</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>3218230.3030303046</c:v>
+                  <c:v>3418930.3030303041</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>3390487.8787878803</c:v>
+                  <c:v>3607224.2424242436</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>3562745.454545456</c:v>
+                  <c:v>3795518.181818183</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>3735003.0303030317</c:v>
+                  <c:v>3983812.1212121225</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>3907260.6060606074</c:v>
+                  <c:v>4172106.0606060619</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>4079518.181818183</c:v>
+                  <c:v>4360400.0000000019</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>4251775.7575757587</c:v>
+                  <c:v>4548693.9393939413</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>4424033.3333333349</c:v>
+                  <c:v>4736987.8787878808</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>4596290.909090911</c:v>
+                  <c:v>4925281.8181818202</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2159,44 +2167,57 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="K15" t="s">
+        <v>63</v>
+      </c>
+      <c r="L15" s="21">
+        <f>L7*$D$10*30</f>
+        <v>18000</v>
+      </c>
+      <c r="M15" s="21">
+        <f>M7*$D$10*30</f>
+        <v>36000</v>
+      </c>
+      <c r="N15" s="21">
+        <f>N7*$D$10*30</f>
+        <v>72000</v>
+      </c>
+      <c r="O15" s="21">
+        <f>O7*$D$10*30</f>
+        <v>108000</v>
+      </c>
+      <c r="P15" s="21">
+        <f>P7*$D$10*30</f>
+        <v>144000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="C16"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="C17"/>
+      <c r="K17" t="s">
         <v>9</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L17" s="9">
         <f>L7*30*$D$10*($D$9*$D$7+$D$8/$B$1)</f>
         <v>47454.545454545463</v>
       </c>
-      <c r="M15" s="9">
+      <c r="M17" s="9">
         <f>M7*30*$D$10*($D$9*$D$7+$D$8/$B$1)</f>
         <v>94909.090909090926</v>
       </c>
-      <c r="N15" s="9">
+      <c r="N17" s="9">
         <f>N7*30*$D$10*($D$9*$D$7+$D$8/$B$1)</f>
         <v>189818.18181818185</v>
       </c>
-      <c r="O15" s="9">
+      <c r="O17" s="9">
         <f>O7*30*$D$10*($D$9*$D$7+$D$8/$B$1)</f>
         <v>284727.27272727276</v>
       </c>
-      <c r="P15" s="9">
+      <c r="P17" s="9">
         <f>P7*30*$D$10*($D$9*$D$7+$D$8/$B$1)</f>
         <v>379636.36363636371</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C16"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C17"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="9"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
@@ -2983,27 +3004,27 @@
         <v>46</v>
       </c>
       <c r="D56" s="20">
-        <v>0</v>
-      </c>
-      <c r="L56" s="17">
-        <f>-$D$56*L15</f>
-        <v>0</v>
-      </c>
-      <c r="M56" s="17">
-        <f t="shared" ref="M56:P56" si="7">-$D$56*M15</f>
-        <v>0</v>
-      </c>
-      <c r="N56" s="17">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="O56" s="17">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P56" s="17">
-        <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.1</v>
+      </c>
+      <c r="L56" s="9">
+        <f>-L15*$D$8/$B$1*$D$56</f>
+        <v>-2045.4545454545457</v>
+      </c>
+      <c r="M56" s="9">
+        <f>-M15*$D$8/$B$1*$D$56</f>
+        <v>-4090.9090909090914</v>
+      </c>
+      <c r="N56" s="9">
+        <f>-N15*$D$8/$B$1*$D$56</f>
+        <v>-8181.8181818181829</v>
+      </c>
+      <c r="O56" s="9">
+        <f>-O15*$D$8/$B$1*$D$56</f>
+        <v>-12272.727272727272</v>
+      </c>
+      <c r="P56" s="9">
+        <f>-P15*$D$8/$B$1*$D$56</f>
+        <v>-16363.636363636366</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
@@ -3014,24 +3035,24 @@
         <v>35</v>
       </c>
       <c r="L58" s="9">
-        <f>-L5*L15</f>
+        <f>-L15*L5*$D$8/$B$1</f>
         <v>0</v>
       </c>
       <c r="M58" s="9">
-        <f>-M5*M15</f>
-        <v>-4745.4545454545469</v>
+        <f>-M15*M5*$D$8/$B$1</f>
+        <v>-2045.4545454545455</v>
       </c>
       <c r="N58" s="9">
-        <f>-N5*N15</f>
-        <v>-18981.818181818187</v>
+        <f>-N15*N5*$D$8/$B$1</f>
+        <v>-8181.818181818182</v>
       </c>
       <c r="O58" s="9">
-        <f>-O5*O15</f>
-        <v>-42709.090909090912</v>
+        <f>-O15*O5*$D$8/$B$1</f>
+        <v>-18409.090909090908</v>
       </c>
       <c r="P58" s="9">
-        <f>-P5*P15</f>
-        <v>-56945.454545454551</v>
+        <f>-P15*P5*$D$8/$B$1</f>
+        <v>-24545.454545454544</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
@@ -3045,24 +3066,24 @@
         <v>36</v>
       </c>
       <c r="L62" s="10">
-        <f>SUM(L15:L60)</f>
-        <v>23108.96464646465</v>
+        <f>SUM(L17:L60)</f>
+        <v>21063.510101010106</v>
       </c>
       <c r="M62" s="10">
-        <f>SUM(M15:M60)</f>
-        <v>47318.055555555591</v>
+        <f>SUM(M17:M60)</f>
+        <v>45927.146464646503</v>
       </c>
       <c r="N62" s="10">
-        <f>SUM(N15:N60)</f>
-        <v>84624.116161616214</v>
+        <f>SUM(N17:N60)</f>
+        <v>87242.297979798052</v>
       </c>
       <c r="O62" s="10">
-        <f>SUM(O15:O60)</f>
-        <v>121205.93434343432</v>
+        <f>SUM(O17:O60)</f>
+        <v>133233.20707070705</v>
       </c>
       <c r="P62" s="10">
-        <f>SUM(P15:P60)</f>
-        <v>167278.66161616161</v>
+        <f>SUM(P17:P60)</f>
+        <v>183315.02525252529</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
@@ -3213,19 +3234,19 @@
       </c>
       <c r="I10" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K10" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M10" s="9">
         <f>SUM(C10:K10)</f>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N10" s="9">
         <f>N9+M10</f>
-        <v>22154.545454545463</v>
+        <v>20109.090909090919</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -3248,19 +3269,19 @@
       </c>
       <c r="I11" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K11" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M11" s="9">
         <f t="shared" ref="M11:M68" si="0">SUM(C11:K11)</f>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N11" s="9">
         <f t="shared" ref="N11:N68" si="1">N10+M11</f>
-        <v>38892.424242424255</v>
+        <v>34801.515151515167</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -3283,19 +3304,19 @@
       </c>
       <c r="I12" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K12" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M12" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N12" s="9">
         <f t="shared" si="1"/>
-        <v>55630.303030303054</v>
+        <v>49493.939393939421</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -3318,19 +3339,19 @@
       </c>
       <c r="I13" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K13" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M13" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N13" s="9">
         <f t="shared" si="1"/>
-        <v>72368.181818181853</v>
+        <v>64186.363636363676</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -3353,19 +3374,19 @@
       </c>
       <c r="I14" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K14" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M14" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N14" s="9">
         <f t="shared" si="1"/>
-        <v>89106.060606060651</v>
+        <v>78878.787878787931</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -3388,19 +3409,19 @@
       </c>
       <c r="I15" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K15" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M15" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N15" s="9">
         <f t="shared" si="1"/>
-        <v>105843.93939393945</v>
+        <v>93571.212121212186</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -3423,19 +3444,19 @@
       </c>
       <c r="I16" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K16" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M16" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N16" s="9">
         <f t="shared" si="1"/>
-        <v>122581.81818181825</v>
+        <v>108263.63636363644</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -3458,19 +3479,19 @@
       </c>
       <c r="I17" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K17" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M17" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N17" s="9">
         <f t="shared" si="1"/>
-        <v>139319.69696969705</v>
+        <v>122956.0606060607</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -3493,19 +3514,19 @@
       </c>
       <c r="I18" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K18" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M18" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N18" s="9">
         <f t="shared" si="1"/>
-        <v>156057.57575757583</v>
+        <v>137648.48484848495</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -3528,19 +3549,19 @@
       </c>
       <c r="I19" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K19" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M19" s="9">
         <f t="shared" si="0"/>
-        <v>16737.878787878795</v>
+        <v>14692.424242424251</v>
       </c>
       <c r="N19" s="9">
         <f t="shared" si="1"/>
-        <v>172795.45454545462</v>
+        <v>152340.9090909092</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -3571,19 +3592,19 @@
       </c>
       <c r="I20" s="9">
         <f>Main!$L$58+Main!$L$56</f>
-        <v>0</v>
+        <v>-2045.4545454545457</v>
       </c>
       <c r="K20" s="9">
-        <f>Main!$L$15</f>
+        <f>Main!$L$17</f>
         <v>47454.545454545463</v>
       </c>
       <c r="M20" s="9">
         <f t="shared" si="0"/>
-        <v>-69800.000000000029</v>
+        <v>-71845.454545454559</v>
       </c>
       <c r="N20" s="9">
         <f t="shared" si="1"/>
-        <v>102995.45454545459</v>
+        <v>80495.454545454646</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -3606,19 +3627,19 @@
       </c>
       <c r="I21" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K21" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M21" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N21" s="9">
         <f t="shared" si="1"/>
-        <v>145242.42424242431</v>
+        <v>121351.51515151527</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -3641,19 +3662,19 @@
       </c>
       <c r="I22" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K22" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M22" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N22" s="9">
         <f t="shared" si="1"/>
-        <v>187489.39393939404</v>
+        <v>162207.57575757589</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -3676,19 +3697,19 @@
       </c>
       <c r="I23" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K23" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M23" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N23" s="9">
         <f t="shared" si="1"/>
-        <v>229736.36363636376</v>
+        <v>203063.63636363653</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -3711,19 +3732,19 @@
       </c>
       <c r="I24" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K24" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M24" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N24" s="9">
         <f t="shared" si="1"/>
-        <v>271983.33333333349</v>
+        <v>243919.69696969714</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -3746,19 +3767,19 @@
       </c>
       <c r="I25" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K25" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M25" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N25" s="9">
         <f t="shared" si="1"/>
-        <v>314230.30303030321</v>
+        <v>284775.75757575774</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -3781,19 +3802,19 @@
       </c>
       <c r="I26" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K26" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M26" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N26" s="9">
         <f t="shared" si="1"/>
-        <v>356477.27272727294</v>
+        <v>325631.81818181835</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -3816,19 +3837,19 @@
       </c>
       <c r="I27" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K27" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M27" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N27" s="9">
         <f t="shared" si="1"/>
-        <v>398724.24242424266</v>
+        <v>366487.87878787896</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -3851,19 +3872,19 @@
       </c>
       <c r="I28" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K28" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M28" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N28" s="9">
         <f t="shared" si="1"/>
-        <v>440971.21212121239</v>
+        <v>407343.93939393957</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
@@ -3886,19 +3907,19 @@
       </c>
       <c r="I29" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K29" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M29" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N29" s="9">
         <f t="shared" si="1"/>
-        <v>483218.18181818211</v>
+        <v>448200.00000000017</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
@@ -3921,19 +3942,19 @@
       </c>
       <c r="I30" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K30" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M30" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N30" s="9">
         <f t="shared" si="1"/>
-        <v>525465.15151515184</v>
+        <v>489056.06060606078</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -3956,19 +3977,19 @@
       </c>
       <c r="I31" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K31" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M31" s="9">
         <f t="shared" si="0"/>
-        <v>42246.969696969718</v>
+        <v>40856.060606060622</v>
       </c>
       <c r="N31" s="9">
         <f t="shared" si="1"/>
-        <v>567712.12121212156</v>
+        <v>529912.12121212145</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -3999,19 +4020,19 @@
       </c>
       <c r="I32" s="9">
         <f>Main!$M$58+Main!$M$56</f>
-        <v>-4745.4545454545469</v>
+        <v>-6136.3636363636369</v>
       </c>
       <c r="K32" s="9">
-        <f>Main!$M$15</f>
+        <f>Main!$M$17</f>
         <v>94909.090909090926</v>
       </c>
       <c r="M32" s="9">
         <f t="shared" si="0"/>
-        <v>-165290.90909090906</v>
+        <v>-166681.81818181818</v>
       </c>
       <c r="N32" s="9">
         <f t="shared" si="1"/>
-        <v>402421.21212121251</v>
+        <v>363230.30303030327</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -4034,19 +4055,19 @@
       </c>
       <c r="I33" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K33" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M33" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N33" s="9">
         <f t="shared" si="1"/>
-        <v>486824.24242424284</v>
+        <v>450251.51515151543</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -4069,19 +4090,19 @@
       </c>
       <c r="I34" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K34" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M34" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N34" s="9">
         <f t="shared" si="1"/>
-        <v>571227.27272727317</v>
+        <v>537272.72727272753</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -4104,19 +4125,19 @@
       </c>
       <c r="I35" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K35" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M35" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N35" s="9">
         <f t="shared" si="1"/>
-        <v>655630.30303030345</v>
+        <v>624293.93939393968</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -4139,19 +4160,19 @@
       </c>
       <c r="I36" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K36" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M36" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N36" s="9">
         <f t="shared" si="1"/>
-        <v>740033.33333333372</v>
+        <v>711315.15151515184</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -4174,19 +4195,19 @@
       </c>
       <c r="I37" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K37" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M37" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N37" s="9">
         <f t="shared" si="1"/>
-        <v>824436.363636364</v>
+        <v>798336.363636364</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -4209,19 +4230,19 @@
       </c>
       <c r="I38" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K38" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M38" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N38" s="9">
         <f t="shared" si="1"/>
-        <v>908839.39393939427</v>
+        <v>885357.57575757615</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -4244,19 +4265,19 @@
       </c>
       <c r="I39" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K39" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M39" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N39" s="9">
         <f t="shared" si="1"/>
-        <v>993242.42424242455</v>
+        <v>972378.78787878831</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -4279,19 +4300,19 @@
       </c>
       <c r="I40" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K40" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M40" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N40" s="9">
         <f t="shared" si="1"/>
-        <v>1077645.4545454548</v>
+        <v>1059400.0000000005</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -4314,19 +4335,19 @@
       </c>
       <c r="I41" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K41" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M41" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N41" s="9">
         <f t="shared" si="1"/>
-        <v>1162048.4848484851</v>
+        <v>1146421.2121212126</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -4349,19 +4370,19 @@
       </c>
       <c r="I42" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K42" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M42" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N42" s="9">
         <f t="shared" si="1"/>
-        <v>1246451.5151515154</v>
+        <v>1233442.4242424248</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -4384,19 +4405,19 @@
       </c>
       <c r="I43" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K43" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M43" s="9">
         <f t="shared" si="0"/>
-        <v>84403.030303030333</v>
+        <v>87021.212121212156</v>
       </c>
       <c r="N43" s="9">
         <f t="shared" si="1"/>
-        <v>1330854.5454545456</v>
+        <v>1320463.6363636369</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -4427,19 +4448,19 @@
       </c>
       <c r="I44" s="9">
         <f>Main!$N$58+Main!$N$56</f>
-        <v>-18981.818181818187</v>
+        <v>-16363.636363636364</v>
       </c>
       <c r="K44" s="9">
-        <f>Main!$N$15</f>
+        <f>Main!$N$17</f>
         <v>189818.18181818185</v>
       </c>
       <c r="M44" s="9">
         <f t="shared" si="0"/>
-        <v>-96134.84848484848</v>
+        <v>-93516.666666666657</v>
       </c>
       <c r="N44" s="9">
         <f t="shared" si="1"/>
-        <v>1234719.6969696973</v>
+        <v>1226946.9696969702</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -4462,19 +4483,19 @@
       </c>
       <c r="I45" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K45" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M45" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N45" s="9">
         <f t="shared" si="1"/>
-        <v>1358304.5454545459</v>
+        <v>1362559.0909090915</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -4497,19 +4518,19 @@
       </c>
       <c r="I46" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K46" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M46" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N46" s="9">
         <f t="shared" si="1"/>
-        <v>1481889.3939393945</v>
+        <v>1498171.2121212129</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -4532,19 +4553,19 @@
       </c>
       <c r="I47" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K47" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M47" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N47" s="9">
         <f t="shared" si="1"/>
-        <v>1605474.2424242431</v>
+        <v>1633783.3333333342</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -4567,19 +4588,19 @@
       </c>
       <c r="I48" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K48" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M48" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N48" s="9">
         <f t="shared" si="1"/>
-        <v>1729059.0909090918</v>
+        <v>1769395.4545454555</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -4602,19 +4623,19 @@
       </c>
       <c r="I49" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K49" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M49" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N49" s="9">
         <f t="shared" si="1"/>
-        <v>1852643.9393939404</v>
+        <v>1905007.5757575769</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -4637,19 +4658,19 @@
       </c>
       <c r="I50" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K50" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M50" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N50" s="9">
         <f t="shared" si="1"/>
-        <v>1976228.787878789</v>
+        <v>2040619.6969696982</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -4672,19 +4693,19 @@
       </c>
       <c r="I51" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K51" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M51" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N51" s="9">
         <f t="shared" si="1"/>
-        <v>2099813.6363636376</v>
+        <v>2176231.8181818193</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
@@ -4707,19 +4728,19 @@
       </c>
       <c r="I52" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K52" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M52" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N52" s="9">
         <f t="shared" si="1"/>
-        <v>2223398.4848484863</v>
+        <v>2311843.9393939404</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -4742,19 +4763,19 @@
       </c>
       <c r="I53" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K53" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M53" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N53" s="9">
         <f t="shared" si="1"/>
-        <v>2346983.3333333349</v>
+        <v>2447456.0606060615</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -4777,19 +4798,19 @@
       </c>
       <c r="I54" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K54" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M54" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N54" s="9">
         <f t="shared" si="1"/>
-        <v>2470568.1818181835</v>
+        <v>2583068.1818181826</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -4812,19 +4833,19 @@
       </c>
       <c r="I55" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K55" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M55" s="9">
         <f t="shared" si="0"/>
-        <v>123584.84848484851</v>
+        <v>135612.12121212124</v>
       </c>
       <c r="N55" s="9">
         <f t="shared" si="1"/>
-        <v>2594153.0303030321</v>
+        <v>2718680.3030303037</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
@@ -4855,19 +4876,19 @@
       </c>
       <c r="I56" s="9">
         <f>Main!$O$58+Main!$O$56</f>
-        <v>-42709.090909090912</v>
+        <v>-30681.81818181818</v>
       </c>
       <c r="K56" s="9">
-        <f>Main!$O$15</f>
+        <f>Main!$O$17</f>
         <v>284727.27272727276</v>
       </c>
       <c r="M56" s="9">
         <f t="shared" si="0"/>
-        <v>-64953.030303030217</v>
+        <v>-52925.757575757452</v>
       </c>
       <c r="N56" s="9">
         <f t="shared" si="1"/>
-        <v>2529200.0000000019</v>
+        <v>2665754.5454545463</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
@@ -4890,19 +4911,19 @@
       </c>
       <c r="I57" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K57" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M57" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N57" s="9">
         <f t="shared" si="1"/>
-        <v>2701457.5757575775</v>
+        <v>2854048.4848484858</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -4925,19 +4946,19 @@
       </c>
       <c r="I58" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K58" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M58" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N58" s="9">
         <f t="shared" si="1"/>
-        <v>2873715.1515151532</v>
+        <v>3042342.4242424252</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
@@ -4960,19 +4981,19 @@
       </c>
       <c r="I59" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K59" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M59" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N59" s="9">
         <f t="shared" si="1"/>
-        <v>3045972.7272727289</v>
+        <v>3230636.3636363647</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -4995,19 +5016,19 @@
       </c>
       <c r="I60" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K60" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M60" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N60" s="9">
         <f t="shared" si="1"/>
-        <v>3218230.3030303046</v>
+        <v>3418930.3030303041</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
@@ -5030,19 +5051,19 @@
       </c>
       <c r="I61" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K61" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M61" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N61" s="9">
         <f t="shared" si="1"/>
-        <v>3390487.8787878803</v>
+        <v>3607224.2424242436</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
@@ -5065,19 +5086,19 @@
       </c>
       <c r="I62" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K62" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M62" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N62" s="9">
         <f t="shared" si="1"/>
-        <v>3562745.454545456</v>
+        <v>3795518.181818183</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
@@ -5100,19 +5121,19 @@
       </c>
       <c r="I63" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K63" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M63" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N63" s="9">
         <f t="shared" si="1"/>
-        <v>3735003.0303030317</v>
+        <v>3983812.1212121225</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
@@ -5135,19 +5156,19 @@
       </c>
       <c r="I64" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K64" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M64" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N64" s="9">
         <f t="shared" si="1"/>
-        <v>3907260.6060606074</v>
+        <v>4172106.0606060619</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
@@ -5170,19 +5191,19 @@
       </c>
       <c r="I65" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K65" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M65" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N65" s="9">
         <f t="shared" si="1"/>
-        <v>4079518.181818183</v>
+        <v>4360400.0000000019</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
@@ -5205,19 +5226,19 @@
       </c>
       <c r="I66" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K66" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M66" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N66" s="9">
         <f t="shared" si="1"/>
-        <v>4251775.7575757587</v>
+        <v>4548693.9393939413</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
@@ -5240,19 +5261,19 @@
       </c>
       <c r="I67" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K67" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M67" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N67" s="9">
         <f t="shared" si="1"/>
-        <v>4424033.3333333349</v>
+        <v>4736987.8787878808</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
@@ -5275,19 +5296,19 @@
       </c>
       <c r="I68" s="9">
         <f>Main!$P$58+Main!$P$56</f>
-        <v>-56945.454545454551</v>
+        <v>-40909.090909090912</v>
       </c>
       <c r="K68" s="9">
-        <f>Main!$P$15</f>
+        <f>Main!$P$17</f>
         <v>379636.36363636371</v>
       </c>
       <c r="M68" s="9">
         <f t="shared" si="0"/>
-        <v>172257.5757575758</v>
+        <v>188293.93939393945</v>
       </c>
       <c r="N68" s="9">
         <f t="shared" si="1"/>
-        <v>4596290.909090911</v>
+        <v>4925281.8181818202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>